<commit_message>
Update order items and prevented items data files
</commit_message>
<xml_diff>
--- a/data/input/prevented_items/drugprevented.xlsx
+++ b/data/input/prevented_items/drugprevented.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,14 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>mnr skin bonetab</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AVIL 6 AMP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix bug from refractoring
</commit_message>
<xml_diff>
--- a/data/input/prevented_items/drugprevented.xlsx
+++ b/data/input/prevented_items/drugprevented.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\prevented_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E983BB5-3F24-42BD-8B84-32C605E443D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F246886-BC9E-4906-9449-5E7D7D36D86E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="303">
   <si>
     <t>كود</t>
   </si>
@@ -634,13 +634,313 @@
   </si>
   <si>
     <t>THYROCARBIN 5MG 50 TABS</t>
+  </si>
+  <si>
+    <t>EUCAL GEL 50 GM</t>
+  </si>
+  <si>
+    <t>DRAVOCAL 120 ML</t>
+  </si>
+  <si>
+    <t>KY GEL PERFECT 85GM</t>
+  </si>
+  <si>
+    <t>EUCAL GEL MASSAGE 30 GM</t>
+  </si>
+  <si>
+    <t>TOUX PROSPERITY SYRUP 120 ML</t>
+  </si>
+  <si>
+    <t>MISHA MULTIVITAMIN SYRUP</t>
+  </si>
+  <si>
+    <t>KIDSOMEAL SYRUP</t>
+  </si>
+  <si>
+    <t>PAINOMOVE TAB</t>
+  </si>
+  <si>
+    <t>HIMAX VIT SYRUP</t>
+  </si>
+  <si>
+    <t>REDGLOB 30 CAPS</t>
+  </si>
+  <si>
+    <t>ROTADANSETRON 4MG/2ML 5 I.M./I.V./INF. AMP.</t>
+  </si>
+  <si>
+    <t>ROTADANSETRON 8MG/2ML 5 I.M./I.V./INF. AMP.</t>
+  </si>
+  <si>
+    <t>DIGEASIA CAPS</t>
+  </si>
+  <si>
+    <t>FEROJUST 30 CAPS</t>
+  </si>
+  <si>
+    <t>VARDENORECT 20 MG 8 TAB</t>
+  </si>
+  <si>
+    <t>LEVOFOXAT 500 MG 5 TABS</t>
+  </si>
+  <si>
+    <t>ACTITRUE MOUTH WASH</t>
+  </si>
+  <si>
+    <t>ACTITRUE INTIMATE FEMININE WASH 200ml</t>
+  </si>
+  <si>
+    <t>ACTITRUE CALAMINE LOTION 100ml</t>
+  </si>
+  <si>
+    <t>ZINCOKID LOTION 120ML</t>
+  </si>
+  <si>
+    <t>well baby spray</t>
+  </si>
+  <si>
+    <t>WELL BABY SYRUP 120ML</t>
+  </si>
+  <si>
+    <t>NIGRA STREP 12LOZENGES</t>
+  </si>
+  <si>
+    <t>ISTIKREMA CREAM</t>
+  </si>
+  <si>
+    <t>SWELLARO 50 GM GEL</t>
+  </si>
+  <si>
+    <t>SALINEX DROPS</t>
+  </si>
+  <si>
+    <t>TRUST SYRUP 120ML</t>
+  </si>
+  <si>
+    <t>unicetamol oral drops for children 15ml</t>
+  </si>
+  <si>
+    <t>Awadist 1000 mg Tab</t>
+  </si>
+  <si>
+    <t>ACETYL-C CORCEPT 20CAPS</t>
+  </si>
+  <si>
+    <t>JUNEL CARE VAG FOAMING SOLUTION 250 ML</t>
+  </si>
+  <si>
+    <t>MEBOLIVIA CREAM</t>
+  </si>
+  <si>
+    <t>FERMED 100MG/5ML 5 AMP</t>
+  </si>
+  <si>
+    <t>VIRECTA PLUS 4 TABS</t>
+  </si>
+  <si>
+    <t>ALC WHITE FIELD DROP</t>
+  </si>
+  <si>
+    <t>diaper oint</t>
+  </si>
+  <si>
+    <t>PREDAPOX 60 MG 6 F.C. TABS</t>
+  </si>
+  <si>
+    <t>pot.permengenete lotion</t>
+  </si>
+  <si>
+    <t>CIPROFLOXMET 500/500MG 20 F.C.TABS.</t>
+  </si>
+  <si>
+    <t>AFERMAX TABS</t>
+  </si>
+  <si>
+    <t>BABY RELIEF 25 MG 10 SUPP.</t>
+  </si>
+  <si>
+    <t>FREE SYRUP</t>
+  </si>
+  <si>
+    <t>BABY RELIFE 12.5 2 STRIPS SUPP</t>
+  </si>
+  <si>
+    <t>AZITANAD 500MG TAB</t>
+  </si>
+  <si>
+    <t>JEPARILON 20 TABS</t>
+  </si>
+  <si>
+    <t>CHEMICETRIZINE 5 MG20 TAB</t>
+  </si>
+  <si>
+    <t>GINSO MAX 30 CAPSULE</t>
+  </si>
+  <si>
+    <t>APPE-RAISE SYRUP 120 ML</t>
+  </si>
+  <si>
+    <t>MIXTANE 30TABS</t>
+  </si>
+  <si>
+    <t>LMODOXACIN 750MG 10 TAB</t>
+  </si>
+  <si>
+    <t>IVYPTO 120 ML SYRUP</t>
+  </si>
+  <si>
+    <t>COBALAMIN DEPOT 5AMP</t>
+  </si>
+  <si>
+    <t>VISCERA SYRUP 120 ML</t>
+  </si>
+  <si>
+    <t>GAMATERN 20 TABS</t>
+  </si>
+  <si>
+    <t>BENDAX TAB</t>
+  </si>
+  <si>
+    <t>RotMOOV 40GM MASSAGE CREAM</t>
+  </si>
+  <si>
+    <t>FAMOTIN 40MG TAB</t>
+  </si>
+  <si>
+    <t>ANTIFLAM 50MG 20TAB</t>
+  </si>
+  <si>
+    <t>C ZINC 30 HARD GELATIN CAPSULES</t>
+  </si>
+  <si>
+    <t>RHINEX ADULT DROPS</t>
+  </si>
+  <si>
+    <t>MOVIGIT 50 MG 30 TAB</t>
+  </si>
+  <si>
+    <t>ADWIFLAM 6 AMP</t>
+  </si>
+  <si>
+    <t>TEMPORAL SYP 60 ML</t>
+  </si>
+  <si>
+    <t>B-MELT 30 INSTANT DISSOLVE TABS</t>
+  </si>
+  <si>
+    <t>UCAL CREAM 50 GM</t>
+  </si>
+  <si>
+    <t>XICLAV 1 GM 14 TABS</t>
+  </si>
+  <si>
+    <t>CRYPTONAZ SUSP</t>
+  </si>
+  <si>
+    <t>CRYPTONAZ 12 TAB</t>
+  </si>
+  <si>
+    <t>Omega RX 60 pieces + Omega 30 pieces offer</t>
+  </si>
+  <si>
+    <t>SILVER SEAS SYR</t>
+  </si>
+  <si>
+    <t>SILVER SEAS CAP</t>
+  </si>
+  <si>
+    <t>BREVY 2.5MG/5ML SYRUP 100 ML</t>
+  </si>
+  <si>
+    <t>BREVY 5 MG 10 F.C. TABS.</t>
+  </si>
+  <si>
+    <t>OMEGACOUGH 120ML SYRUP</t>
+  </si>
+  <si>
+    <t>ZANDROS 20 CAPS</t>
+  </si>
+  <si>
+    <t>MOVENTOR 20TAB</t>
+  </si>
+  <si>
+    <t>FLUOROCARE ORAL GEL</t>
+  </si>
+  <si>
+    <t>PREMAPRESS 30 TABLETS</t>
+  </si>
+  <si>
+    <t>OSTEPRESS 30 TAB</t>
+  </si>
+  <si>
+    <t>PRINU 15 SACHETS</t>
+  </si>
+  <si>
+    <t>RICOGENEX 10 SACHET</t>
+  </si>
+  <si>
+    <t>PROTOPAN 40 MG 21 CAPS</t>
+  </si>
+  <si>
+    <t>pressrol gel 50 gm</t>
+  </si>
+  <si>
+    <t>NEEROMELLA PLUS DIAPER CREAM</t>
+  </si>
+  <si>
+    <t>NEEROMELLA 30 GM CREAM</t>
+  </si>
+  <si>
+    <t>AZITHROMYCIN AUG 500 MG 6 TAB</t>
+  </si>
+  <si>
+    <t>FEVONOXOL 1 GM 20 TABLETS</t>
+  </si>
+  <si>
+    <t>ULTRAHUMIDIN CREAM</t>
+  </si>
+  <si>
+    <t>JEPARILON 10 MG 10 CHEW. TABS</t>
+  </si>
+  <si>
+    <t>moventor 30 tab</t>
+  </si>
+  <si>
+    <t>AZITHROMYCIN-AUG 500 MG 6 F.C.TABS</t>
+  </si>
+  <si>
+    <t>IMMUNO-MASH 30 F.C.TABS</t>
+  </si>
+  <si>
+    <t>RIOPANOX 160 ML LIQUID</t>
+  </si>
+  <si>
+    <t>BABY RELIEF 25 MG 10 SUPP</t>
+  </si>
+  <si>
+    <t>ZYMAGALLINE TAB</t>
+  </si>
+  <si>
+    <t>EUCAL HERBAL MASSAGE GEL 30 GM</t>
+  </si>
+  <si>
+    <t>SILVER SEAS SYRUP</t>
+  </si>
+  <si>
+    <t>EUCAL CREAM 50 GM</t>
+  </si>
+  <si>
+    <t>ELMODOXACIN 750MG 10 TAB</t>
+  </si>
+  <si>
+    <t>TADANERFI 20MG 4FILM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -654,16 +954,47 @@
       <name val="Noto Sans Devanagari"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF6AA84F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -671,13 +1002,79 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -874,7 +1271,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B197"/>
+  <dimension ref="A1:B313"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="31.85546875" customWidth="1"/>
@@ -2448,12 +2845,592 @@
         <v>200</v>
       </c>
     </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>201</v>
       </c>
       <c r="B197" t="s">
         <v>202</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B198" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B199" s="3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B200" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B201" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B202" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B203" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B204" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B205" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B206" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B207" s="3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B208" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="209" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B209" s="3" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="210" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B210" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="211" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B211" s="3" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="212" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B212" s="3" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="213" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B213" s="3" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="214" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B214" s="3" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="215" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B215" s="2" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="216" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B216" s="3" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="217" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B217" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="218" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B218" s="3" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="219" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B219" s="3" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="220" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B220" s="3" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="221" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B221" s="3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="222" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B222" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="223" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B223" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="224" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B224" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="225" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B225" s="3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="226" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B226" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="227" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B227" s="3" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="228" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B228" s="3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="229" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B229" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="230" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B230" s="3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="231" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B231" s="3" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="232" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B232" s="3" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="233" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B233" s="3" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="234" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B234" s="3" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="235" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B235" s="3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="236" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B236" s="3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="237" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B237" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="238" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B238" s="3" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="239" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B239" s="2" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="240" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B240" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="241" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B241" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="242" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B242" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="243" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B243" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="244" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B244" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="245" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B245" s="2" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="246" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B246" s="2" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="247" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B247" s="2" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="248" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B248" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="249" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B249" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="250" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B250" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="251" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B251" s="2" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="252" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B252" s="3" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="253" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B253" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="254" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B254" s="3" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="255" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B255" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="256" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B256" s="3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="257" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B257" s="3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="258" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B258" s="3" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="259" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B259" s="3" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="260" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B260" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="261" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B261" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="262" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B262" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="263" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B263" s="3" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="264" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B264" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="265" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B265" s="3" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="266" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B266" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="267" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B267" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="268" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B268" s="3" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="269" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B269" s="2" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="270" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B270" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="271" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B271" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="272" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B272" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="273" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B273" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="274" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B274" s="2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="275" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B275" s="2" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="276" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B276" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="277" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B277" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="278" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B278" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="279" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B279" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="280" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B280" s="2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="281" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B281" s="3" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="282" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B282" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="283" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B283" s="3" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="284" spans="2:2" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B284" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="285" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B285" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="286" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B286" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="287" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B287" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="288" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B288" s="2" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="289" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B289" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="290" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B290" s="2" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="291" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B291" s="2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="292" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B292" s="2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="293" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B293" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="294" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B294" s="3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="295" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B295" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="296" spans="2:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B296" s="4" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="297" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B297" s="5" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="298" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B298" s="6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="299" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B299" s="6" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="300" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B300" s="6" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="301" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B301" s="6" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="302" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B302" s="6" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="303" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B303" s="6" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="304" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B304" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="305" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B305" s="6" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="306" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B306" s="5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="307" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B307" s="6" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="308" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B308" s="5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="309" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B309" s="6" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="310" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B310" s="6" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="311" spans="2:2" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B311" s="6" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="312" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B312" s="7" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="313" spans="2:2" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B313" s="8" t="s">
+        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
solve co avazir problem
</commit_message>
<xml_diff>
--- a/data/input/prevented_items/drugprevented.xlsx
+++ b/data/input/prevented_items/drugprevented.xlsx
@@ -8,15 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\prevented_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFEE28A7-1B3E-492B-B80B-0F80A2199820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D053A0-0FD4-424A-ADBD-8FEEF0E77357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-10410" windowWidth="16440" windowHeight="28320" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -25,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="457">
   <si>
     <t>كود</t>
   </si>
@@ -1042,13 +1053,367 @@
   </si>
   <si>
     <t>G T N MEGA STAR</t>
+  </si>
+  <si>
+    <t>79407</t>
+  </si>
+  <si>
+    <t>LILI FEMININE WASH 250ML</t>
+  </si>
+  <si>
+    <t>86113</t>
+  </si>
+  <si>
+    <t>DEMAS D3 10.000 I.U 30 TABS</t>
+  </si>
+  <si>
+    <t>47262</t>
+  </si>
+  <si>
+    <t>PECTOL bluo+vit c</t>
+  </si>
+  <si>
+    <t>88907</t>
+  </si>
+  <si>
+    <t>TETRA CARE HAIR SHAMPOO 200 ML</t>
+  </si>
+  <si>
+    <t>59550</t>
+  </si>
+  <si>
+    <t>EXTRAGESIC 400 MG 20 TAB</t>
+  </si>
+  <si>
+    <t>73934</t>
+  </si>
+  <si>
+    <t>DANSET 4 MG  3 AMP/2 ML</t>
+  </si>
+  <si>
+    <t>91191</t>
+  </si>
+  <si>
+    <t>SANSO D3 PLUS 28 TAB</t>
+  </si>
+  <si>
+    <t>90845</t>
+  </si>
+  <si>
+    <t>LACTASE 750 DROPS 15ML</t>
+  </si>
+  <si>
+    <t>57376</t>
+  </si>
+  <si>
+    <t>LIPITOR 40 MG 14 TAB</t>
+  </si>
+  <si>
+    <t>FERTINA BONAVIDEA 30 HARD CAPSULES</t>
+  </si>
+  <si>
+    <t>ACELIOFINAZ 100 MG 20 F.C. TAB</t>
+  </si>
+  <si>
+    <t>ADWIFLOXACEN 400 MG 7 TABS</t>
+  </si>
+  <si>
+    <t>AIRONYL 2.5 MG 20 TAB</t>
+  </si>
+  <si>
+    <t>ALZMENDA 10 MG ORAL DROPS</t>
+  </si>
+  <si>
+    <t>ARTICU-SAFE 30 CAP</t>
+  </si>
+  <si>
+    <t>ASPIRIN-CHEMIPHARM 75 MG 30 CHEW.TABS.</t>
+  </si>
+  <si>
+    <t>BOWELOCARE ORAL DROPS 15 ML</t>
+  </si>
+  <si>
+    <t>BRONCHO-VAXOM SACHETS</t>
+  </si>
+  <si>
+    <t>CARNITOL 500 MG 30 CAP</t>
+  </si>
+  <si>
+    <t>CIPROCIN EYE OINTMENT 5 GM</t>
+  </si>
+  <si>
+    <t>COLLABUILD PLUS 30 TABS</t>
+  </si>
+  <si>
+    <t>CORNEFRESH 15MG EYE DROPS</t>
+  </si>
+  <si>
+    <t>COXRITOR 120 MG 10 F.C.TABS</t>
+  </si>
+  <si>
+    <t>CUIDADO 30 TABS</t>
+  </si>
+  <si>
+    <t>CYSTINOL CAP</t>
+  </si>
+  <si>
+    <t>DELPANTO 20 MG  CAP</t>
+  </si>
+  <si>
+    <t>DEXKETO CARE 25 MG 30 TAB</t>
+  </si>
+  <si>
+    <t>DISPERCAM 20MG TAB</t>
+  </si>
+  <si>
+    <t>DOLABACTIN 400MG 5TAB</t>
+  </si>
+  <si>
+    <t>DOLPHIN - K 75MG 6 AMP</t>
+  </si>
+  <si>
+    <t>EAZEX-LINE GEL 30 GM</t>
+  </si>
+  <si>
+    <t>EBASTINE-BORG 10MG 10TABS</t>
+  </si>
+  <si>
+    <t>ENERGY SERUM WITH ARGAN OIL 100 ML</t>
+  </si>
+  <si>
+    <t>EPIFENAC 25MG SUPP</t>
+  </si>
+  <si>
+    <t>EPIRAZOLE CAP</t>
+  </si>
+  <si>
+    <t>ESOGERDAZOLE 40 MG MG DR 14 CAP</t>
+  </si>
+  <si>
+    <t>Esomeprazole eva 20 mg 10 cap</t>
+  </si>
+  <si>
+    <t>FLORAGESTIVE IRON 30CAP</t>
+  </si>
+  <si>
+    <t>FLUROFLOX 400 mg 10 TAB</t>
+  </si>
+  <si>
+    <t>GANTOLIEF 50 MG 30 F.C.TABS.</t>
+  </si>
+  <si>
+    <t>GASTRODOMINA 20MG 20 TAB</t>
+  </si>
+  <si>
+    <t>GATYXEL 0.3 % EYE DROPS 5 ML</t>
+  </si>
+  <si>
+    <t>ACNE FREE CREAM 30 GM</t>
+  </si>
+  <si>
+    <t>medicolon tab</t>
+  </si>
+  <si>
+    <t>volvaro oral gel 20gm</t>
+  </si>
+  <si>
+    <t>MIOPAN SYRUP</t>
+  </si>
+  <si>
+    <t>AUGRAM 228.5 60ML SYRUP</t>
+  </si>
+  <si>
+    <t>GIT 20 CAP</t>
+  </si>
+  <si>
+    <t>HEROXACIN 500MG 10 TABS</t>
+  </si>
+  <si>
+    <t>HI-COOL MASSAGE CREAM 50 GM</t>
+  </si>
+  <si>
+    <t>INFECTOCURE 250MG 14TABS</t>
+  </si>
+  <si>
+    <t>JOVEMED B12 - 1000 MCG 30 SUBLINGUAL TABS.</t>
+  </si>
+  <si>
+    <t>KAST 5 MG 14TAB</t>
+  </si>
+  <si>
+    <t>KETOLGIN AMP</t>
+  </si>
+  <si>
+    <t>KLACID 250 MG 14 F.C. TABS</t>
+  </si>
+  <si>
+    <t>L-CARNITINE ZINC  30 CAP</t>
+  </si>
+  <si>
+    <t>LANTANON CAP</t>
+  </si>
+  <si>
+    <t>MARCOTRAVIN 120MG 30 CAPS</t>
+  </si>
+  <si>
+    <t>MEDIOSTEO TAB</t>
+  </si>
+  <si>
+    <t>NORFLEX 100 MG 20 TABS</t>
+  </si>
+  <si>
+    <t>NOTRIPROX 15 G CREAM</t>
+  </si>
+  <si>
+    <t>ORCHACIN DROPS</t>
+  </si>
+  <si>
+    <t>OXYPOL EYE OINT</t>
+  </si>
+  <si>
+    <t>PANTOPI 20 MG 20 TAB</t>
+  </si>
+  <si>
+    <t>PREDNISOLONE EVAPHARMA 20NG</t>
+  </si>
+  <si>
+    <t>PROSTACURE CAP</t>
+  </si>
+  <si>
+    <t>ROOTAGE OIL</t>
+  </si>
+  <si>
+    <t>S.M.R 20TAB</t>
+  </si>
+  <si>
+    <t>SLEEVAR PREGNA 30CAP</t>
+  </si>
+  <si>
+    <t>STATURIC 80 MG 30TAB</t>
+  </si>
+  <si>
+    <t>STEADYFUTAL 16 MG 60 TAB.</t>
+  </si>
+  <si>
+    <t>SUPER GINKO 60 MG 20 CAP</t>
+  </si>
+  <si>
+    <t>TARIFLOX 200 MG 10 TAB</t>
+  </si>
+  <si>
+    <t>TEBOFORTIN 40 MG ORAL DROPS</t>
+  </si>
+  <si>
+    <t>TRANEX 500 MG 30 TAB</t>
+  </si>
+  <si>
+    <t>TRENCEDIA 550 MG 10 TAB</t>
+  </si>
+  <si>
+    <t>UNOVIT SYRUP</t>
+  </si>
+  <si>
+    <t>VIAVAG  25MG 10 TAB</t>
+  </si>
+  <si>
+    <t>XILOPRED 4MG 20TABS</t>
+  </si>
+  <si>
+    <t>acanthaprop eye 10ml</t>
+  </si>
+  <si>
+    <t>b12 sano pharma 30 s tab</t>
+  </si>
+  <si>
+    <t>clear air 7 sachets 4mg</t>
+  </si>
+  <si>
+    <t>demancortil 2 mg amp</t>
+  </si>
+  <si>
+    <t>keflex 500gm 12 taps</t>
+  </si>
+  <si>
+    <t>kevork 500 mg 10 tab</t>
+  </si>
+  <si>
+    <t>lantopep 60mg 14 tab</t>
+  </si>
+  <si>
+    <t>رواكد</t>
+  </si>
+  <si>
+    <t>تصحيح تكويد</t>
+  </si>
+  <si>
+    <t>اكسبير</t>
+  </si>
+  <si>
+    <t>طلب خاص</t>
+  </si>
+  <si>
+    <t>بريفير</t>
+  </si>
+  <si>
+    <t>L-CARNITINE ZINC  30 CAP</t>
+  </si>
+  <si>
+    <t>VIAVAG  25MG 10 TAB</t>
+  </si>
+  <si>
+    <t>ALERGAWAY 5MG 20 DIS.TAB</t>
+  </si>
+  <si>
+    <t>MENESTRO 1000 MG 20 CAPS</t>
+  </si>
+  <si>
+    <t>FEMAPENT 2.5MG 14 TABS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">هناك صنف اخر منه </t>
+  </si>
+  <si>
+    <t>MAALOX SUSP 250 ML</t>
+  </si>
+  <si>
+    <t>MAALOX PLUS FAST 180ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">صنفين بنفس السعر وله كودين موقوف لحين تصحيحه من المخزن </t>
+  </si>
+  <si>
+    <t xml:space="preserve">مش عوزينه </t>
+  </si>
+  <si>
+    <t xml:space="preserve">تاريخ </t>
+  </si>
+  <si>
+    <t>NEXIUM 40 MG 28 TABS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اكسبير </t>
+  </si>
+  <si>
+    <t>NANYMOM 30 TAB</t>
+  </si>
+  <si>
+    <t>LIDOCAINE 1 1 AMP 2 ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">تعليمات المدير </t>
+  </si>
+  <si>
+    <t>ROSUCHOLEST 20MG 20 TAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مفيش منه 20 قرص </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1081,8 +1446,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1104,6 +1475,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1148,7 +1525,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -1166,9 +1543,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1365,10 +1744,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B373"/>
+  <dimension ref="A1:C502"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="65.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.5" x14ac:dyDescent="0.35">
@@ -2907,7 +3287,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>92794</v>
       </c>
@@ -2915,7 +3295,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>77847</v>
       </c>
@@ -2923,7 +3303,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>53812</v>
       </c>
@@ -2931,7 +3311,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>92957</v>
       </c>
@@ -2939,7 +3319,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>201</v>
       </c>
@@ -2947,651 +3327,1023 @@
         <v>202</v>
       </c>
     </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B198" s="3" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C198" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B199" s="4" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C199" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B200" s="3" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C200" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B201" s="3" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C201" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B202" s="3" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C202" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B203" s="4" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C203" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B204" s="4" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C204" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B205" s="4" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C205" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B206" s="4" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C206" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B207" s="4" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C207" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B208" s="4" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C208" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="209" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B209" s="4" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C209" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="210" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B210" s="4" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C210" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="211" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B211" s="4" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C211" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="212" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B212" s="4" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C212" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="213" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B213" s="4" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C213" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="214" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B214" s="4" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C214" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="215" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B215" s="3" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C215" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="216" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B216" s="4" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C216" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="217" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B217" s="4" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C217" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="218" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B218" s="4" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C218" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="219" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B219" s="4" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C219" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="220" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B220" s="4" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C220" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="221" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B221" s="4" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C221" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="222" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B222" s="4" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C222" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="223" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B223" s="4" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C223" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="224" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B224" s="3" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C224" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="225" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B225" s="4" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C225" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="226" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B226" s="3" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C226" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="227" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B227" s="4" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C227" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="228" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B228" s="4" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C228" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="229" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B229" s="4" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C229" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="230" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B230" s="4" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C230" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="231" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B231" s="4" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C231" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="232" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B232" s="4" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C232" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="233" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B233" s="4" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C233" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="234" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B234" s="4" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C234" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="235" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B235" s="4" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C235" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="236" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B236" s="4" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C236" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="237" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B237" s="4" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C237" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="238" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B238" s="4" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C238" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="239" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B239" s="3" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C239" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="240" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B240" s="4" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C240" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="241" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B241" s="4" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C241" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="242" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B242" s="4" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C242" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="243" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B243" s="3" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C243" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="244" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B244" s="4" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C244" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="245" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B245" s="3" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C245" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="246" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B246" s="3" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C246" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="247" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B247" s="3" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C247" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="248" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B248" s="3" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C248" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="249" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B249" s="3" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C249" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="250" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B250" s="4" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C250" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="251" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B251" s="3" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C251" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="252" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B252" s="4" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C252" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="253" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B253" s="3" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C253" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="254" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B254" s="4" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C254" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="255" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B255" s="4" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C255" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="256" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B256" s="4" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C256" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="257" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B257" s="4" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C257" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="258" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B258" s="4" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C258" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="259" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B259" s="4" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C259" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="260" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B260" s="3" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C260" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="261" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B261" s="4" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C261" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="262" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B262" s="4" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C262" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="263" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B263" s="4" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C263" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="264" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B264" s="4" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C264" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="265" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B265" s="4" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C265" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="266" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B266" s="4" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C266" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="267" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B267" s="4" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C267" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="268" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B268" s="4" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C268" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="269" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B269" s="3" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C269" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="270" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B270" s="4" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C270" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="271" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B271" s="4" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C271" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="272" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B272" s="4" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C272" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="273" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B273" s="4" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C273" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="274" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B274" s="3" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C274" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="275" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B275" s="3" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C275" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="276" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B276" s="3" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C276" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="277" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B277" s="3" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C277" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="278" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B278" s="4" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C278" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="279" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B279" s="3" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C279" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="280" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B280" s="3" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C280" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="281" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B281" s="4" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C281" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="282" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B282" s="4" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C282" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="283" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B283" s="4" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C283" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="284" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B284" s="4" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C284" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="285" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B285" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C285" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="286" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B286" s="3" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C286" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="287" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B287" s="3" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C287" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="288" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B288" s="3" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C288" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="289" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B289" s="3" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C289" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="290" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B290" s="3" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C290" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="291" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B291" s="3" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C291" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="292" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B292" s="3" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C292" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="293" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B293" s="3" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C293" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="294" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B294" s="4" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C294" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="295" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B295" s="3" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C295" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="296" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B296" s="3" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="297" spans="2:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C296" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="297" spans="2:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B297" s="5" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="298" spans="2:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C297" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="298" spans="2:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B298" s="6" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="299" spans="2:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C298" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="299" spans="2:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B299" s="6" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="300" spans="2:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C299" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="300" spans="2:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B300" s="6" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="301" spans="2:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C300" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="301" spans="2:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B301" s="6" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="302" spans="2:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C301" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="302" spans="2:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B302" s="6" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="303" spans="2:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C302" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="303" spans="2:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B303" s="6" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="304" spans="2:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C303" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="304" spans="2:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B304" s="5" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="305" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C304" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B305" s="6" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="306" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C305" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B306" s="5" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="307" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C306" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B307" s="6" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="308" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C307" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B308" s="5" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="309" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C308" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B309" s="6" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="310" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C309" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B310" s="6" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="311" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C310" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B311" s="6" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="312" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C311" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B312" s="6" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="313" spans="1:2" ht="18" x14ac:dyDescent="0.25">
+      <c r="C312" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" ht="18" x14ac:dyDescent="0.25">
       <c r="B313" s="6" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C313" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>303</v>
       </c>
       <c r="B314" s="2" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="315" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C314" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>305</v>
       </c>
       <c r="B315" s="2" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="316" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C315" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>307</v>
       </c>
       <c r="B316" s="2" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="317" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C316" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>309</v>
       </c>
       <c r="B317" s="2" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="318" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C317" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>311</v>
       </c>
       <c r="B318" s="2" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="319" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C318" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>313</v>
       </c>
       <c r="B319" s="2" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="320" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C319" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>315</v>
       </c>
       <c r="B320" s="2" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C320" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>317</v>
       </c>
       <c r="B321" s="2" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C321" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322">
         <v>86783</v>
       </c>
@@ -3599,7 +4351,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="323" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A323">
         <v>89070</v>
       </c>
@@ -3607,7 +4359,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="324" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A324">
         <v>48304</v>
       </c>
@@ -3615,7 +4367,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A325">
         <v>49745</v>
       </c>
@@ -3623,7 +4375,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="326" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A326">
         <v>83356</v>
       </c>
@@ -3631,7 +4383,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="327" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A327">
         <v>74752</v>
       </c>
@@ -3639,7 +4391,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A328">
         <v>88451</v>
       </c>
@@ -3647,7 +4399,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="329" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A329">
         <v>88084</v>
       </c>
@@ -3655,7 +4407,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A330">
         <v>91865</v>
       </c>
@@ -3663,7 +4415,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="331" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A331">
         <v>90354</v>
       </c>
@@ -3671,7 +4423,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A332">
         <v>72845</v>
       </c>
@@ -3679,7 +4431,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="333" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A333">
         <v>80145</v>
       </c>
@@ -3687,7 +4439,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="334" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A334">
         <v>81210</v>
       </c>
@@ -3695,7 +4447,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="335" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A335">
         <v>92916</v>
       </c>
@@ -3703,7 +4455,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="336" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A336">
         <v>75077</v>
       </c>
@@ -3839,7 +4591,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="353" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A353">
         <v>82769</v>
       </c>
@@ -3847,7 +4599,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="354" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A354">
         <v>51306</v>
       </c>
@@ -3855,7 +4607,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="355" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
         <v>330</v>
       </c>
@@ -3863,7 +4615,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="356" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A356">
         <v>78132</v>
       </c>
@@ -3871,7 +4623,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="357" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A357">
         <v>9422</v>
       </c>
@@ -3879,7 +4631,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="358" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A358">
         <v>92496</v>
       </c>
@@ -3887,7 +4639,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="359" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A359">
         <v>92139</v>
       </c>
@@ -3895,7 +4647,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="360" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A360">
         <v>53812</v>
       </c>
@@ -3903,7 +4655,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="361" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A361">
         <v>66760</v>
       </c>
@@ -3911,57 +4663,1517 @@
         <v>335</v>
       </c>
     </row>
-    <row r="362" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B362" s="2" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="363" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C362" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="363" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B363" s="2" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="364" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C363" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="364" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B364" s="2" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="365" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C364" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="365" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B365" s="7" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="366" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A366" s="8"/>
-      <c r="B366" s="8"/>
-    </row>
-    <row r="367" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A367" s="8"/>
-      <c r="B367" s="8"/>
-    </row>
-    <row r="368" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A368" s="9"/>
-      <c r="B368" s="9"/>
-    </row>
-    <row r="369" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A369" s="8"/>
-      <c r="B369" s="8"/>
-    </row>
-    <row r="370" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A370" s="8"/>
-      <c r="B370" s="8"/>
-    </row>
-    <row r="371" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A371" s="8"/>
-      <c r="B371" s="8"/>
-    </row>
-    <row r="372" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A372" s="8"/>
-      <c r="B372" s="8"/>
-    </row>
-    <row r="373" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A373" s="8"/>
-      <c r="B373" s="8"/>
+      <c r="C365" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="366" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A366" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="B366" s="8" t="s">
+        <v>340</v>
+      </c>
+      <c r="C366" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="367" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A367" t="s">
+        <v>341</v>
+      </c>
+      <c r="B367" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="368" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A368" t="s">
+        <v>343</v>
+      </c>
+      <c r="B368" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="369" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A369" t="s">
+        <v>345</v>
+      </c>
+      <c r="B369" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="370" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A370" t="s">
+        <v>347</v>
+      </c>
+      <c r="B370" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="371" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A371" t="s">
+        <v>349</v>
+      </c>
+      <c r="B371" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="372" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A372" t="s">
+        <v>351</v>
+      </c>
+      <c r="B372" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="373" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A373" t="s">
+        <v>353</v>
+      </c>
+      <c r="B373" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="374" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A374" t="s">
+        <v>355</v>
+      </c>
+      <c r="B374" t="s">
+        <v>356</v>
+      </c>
+      <c r="C374" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A375">
+        <v>49745</v>
+      </c>
+      <c r="B375" t="s">
+        <v>38</v>
+      </c>
+      <c r="C375" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="376" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A376">
+        <v>49745</v>
+      </c>
+      <c r="B376" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="377" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A377" s="9">
+        <v>86478</v>
+      </c>
+      <c r="B377" s="9" t="s">
+        <v>358</v>
+      </c>
+      <c r="C377" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="378" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A378" s="9">
+        <v>87065</v>
+      </c>
+      <c r="B378" s="9" t="s">
+        <v>359</v>
+      </c>
+      <c r="C378" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="379" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A379" s="9">
+        <v>5953</v>
+      </c>
+      <c r="B379" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="C379" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="380" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A380" s="9">
+        <v>60587</v>
+      </c>
+      <c r="B380" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="C380" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="381" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A381" s="9">
+        <v>74102</v>
+      </c>
+      <c r="B381" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="C381" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="382" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A382" s="9">
+        <v>88301</v>
+      </c>
+      <c r="B382" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="C382" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A383" s="9">
+        <v>92823</v>
+      </c>
+      <c r="B383" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C383" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A384" s="9">
+        <v>81194</v>
+      </c>
+      <c r="B384" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="C384" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="385" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A385" s="9">
+        <v>47526</v>
+      </c>
+      <c r="B385" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="C385" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="386" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A386" s="9">
+        <v>75500</v>
+      </c>
+      <c r="B386" s="9" t="s">
+        <v>366</v>
+      </c>
+      <c r="C386" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="387" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A387" s="9">
+        <v>21246</v>
+      </c>
+      <c r="B387" s="9" t="s">
+        <v>367</v>
+      </c>
+      <c r="C387" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="388" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A388" s="9">
+        <v>92691</v>
+      </c>
+      <c r="B388" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="C388" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="389" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A389" s="9">
+        <v>82161</v>
+      </c>
+      <c r="B389" s="9" t="s">
+        <v>369</v>
+      </c>
+      <c r="C389" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="390" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A390" s="9">
+        <v>88829</v>
+      </c>
+      <c r="B390" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="C390" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="391" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A391" s="9">
+        <v>90318</v>
+      </c>
+      <c r="B391" s="9" t="s">
+        <v>371</v>
+      </c>
+      <c r="C391" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="392" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A392" s="9">
+        <v>48092</v>
+      </c>
+      <c r="B392" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="C392" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="393" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A393" s="9">
+        <v>29208</v>
+      </c>
+      <c r="B393" s="9" t="s">
+        <v>373</v>
+      </c>
+      <c r="C393" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A394" s="9">
+        <v>75410</v>
+      </c>
+      <c r="B394" s="9" t="s">
+        <v>374</v>
+      </c>
+      <c r="C394" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="395" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A395" s="9">
+        <v>21009</v>
+      </c>
+      <c r="B395" s="9" t="s">
+        <v>375</v>
+      </c>
+      <c r="C395" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="396" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A396" s="9">
+        <v>74847</v>
+      </c>
+      <c r="B396" s="9" t="s">
+        <v>376</v>
+      </c>
+      <c r="C396" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="397" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A397" s="9">
+        <v>46762</v>
+      </c>
+      <c r="B397" s="9" t="s">
+        <v>377</v>
+      </c>
+      <c r="C397" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="398" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A398" s="9">
+        <v>154651</v>
+      </c>
+      <c r="B398" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="C398" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="399" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A399" s="9">
+        <v>81914</v>
+      </c>
+      <c r="B399" s="9" t="s">
+        <v>379</v>
+      </c>
+      <c r="C399" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="400" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A400" s="9">
+        <v>44106</v>
+      </c>
+      <c r="B400" s="9" t="s">
+        <v>380</v>
+      </c>
+      <c r="C400" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="401" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A401" s="9">
+        <v>47535</v>
+      </c>
+      <c r="B401" s="9" t="s">
+        <v>381</v>
+      </c>
+      <c r="C401" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="402" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A402" s="9">
+        <v>1576</v>
+      </c>
+      <c r="B402" s="9" t="s">
+        <v>382</v>
+      </c>
+      <c r="C402" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="403" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A403" s="9">
+        <v>68762</v>
+      </c>
+      <c r="B403" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="C403" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="404" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A404" s="9">
+        <v>92091</v>
+      </c>
+      <c r="B404" s="9" t="s">
+        <v>384</v>
+      </c>
+      <c r="C404" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="405" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A405" s="9">
+        <v>90952</v>
+      </c>
+      <c r="B405" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="C405" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="406" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A406" s="9">
+        <v>84597</v>
+      </c>
+      <c r="B406" s="9" t="s">
+        <v>386</v>
+      </c>
+      <c r="C406" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="407" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A407" s="9">
+        <v>79608</v>
+      </c>
+      <c r="B407" s="9" t="s">
+        <v>387</v>
+      </c>
+      <c r="C407" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="408" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A408" s="9">
+        <v>17389</v>
+      </c>
+      <c r="B408" s="9" t="s">
+        <v>388</v>
+      </c>
+      <c r="C408" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="409" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A409" s="9">
+        <v>57777</v>
+      </c>
+      <c r="B409" s="9" t="s">
+        <v>389</v>
+      </c>
+      <c r="C409" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="410" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A410" s="9">
+        <v>4350</v>
+      </c>
+      <c r="B410" s="9" t="s">
+        <v>390</v>
+      </c>
+      <c r="C410" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="411" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A411" s="9">
+        <v>91037</v>
+      </c>
+      <c r="B411" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="C411" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="412" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A412" s="9">
+        <v>89685</v>
+      </c>
+      <c r="B412" s="9" t="s">
+        <v>392</v>
+      </c>
+      <c r="C412" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="413" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A413" s="9">
+        <v>90631</v>
+      </c>
+      <c r="B413" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="C413" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="414" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A414" s="9">
+        <v>23128</v>
+      </c>
+      <c r="B414" s="9" t="s">
+        <v>393</v>
+      </c>
+      <c r="C414" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A415" s="9">
+        <v>79530</v>
+      </c>
+      <c r="B415" s="9" t="s">
+        <v>394</v>
+      </c>
+      <c r="C415" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="416" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A416" s="9">
+        <v>79530</v>
+      </c>
+      <c r="B416" s="9" t="s">
+        <v>394</v>
+      </c>
+      <c r="C416" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="417" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A417" s="9">
+        <v>23302</v>
+      </c>
+      <c r="B417" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="C417" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="418" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A418" s="9">
+        <v>85884</v>
+      </c>
+      <c r="B418" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="C418" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="419" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A419" s="9">
+        <v>49579</v>
+      </c>
+      <c r="B419" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="C419" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="420" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A420" s="9">
+        <v>82381</v>
+      </c>
+      <c r="B420" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="C420" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="421" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A421" s="9">
+        <v>92725</v>
+      </c>
+      <c r="B421" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="C421" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="422" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A422" s="9">
+        <v>53470</v>
+      </c>
+      <c r="B422" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="C422" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="423" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A423" s="9">
+        <v>4522</v>
+      </c>
+      <c r="B423" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="C423" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="424" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A424" s="9">
+        <v>74023</v>
+      </c>
+      <c r="B424" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="C424" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="425" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A425" s="9">
+        <v>92743</v>
+      </c>
+      <c r="B425" s="9" t="s">
+        <v>403</v>
+      </c>
+      <c r="C425" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="426" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A426" s="9">
+        <v>21483</v>
+      </c>
+      <c r="B426" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="C426" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="427" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A427" s="9">
+        <v>80802</v>
+      </c>
+      <c r="B427" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="C427" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="428" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A428" s="9">
+        <v>91036</v>
+      </c>
+      <c r="B428" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="C428" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="429" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A429" s="9">
+        <v>1188</v>
+      </c>
+      <c r="B429" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="C429" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="430" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A430" s="9">
+        <v>84778</v>
+      </c>
+      <c r="B430" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="C430" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="431" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A431" s="9">
+        <v>18096</v>
+      </c>
+      <c r="B431" s="9" t="s">
+        <v>409</v>
+      </c>
+      <c r="C431" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="432" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A432" s="9">
+        <v>17699</v>
+      </c>
+      <c r="B432" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="C432" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="433" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A433" s="9">
+        <v>65983</v>
+      </c>
+      <c r="B433" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="C433" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="434" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A434" s="9">
+        <v>90949</v>
+      </c>
+      <c r="B434" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="C434" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="435" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A435" s="9">
+        <v>8784</v>
+      </c>
+      <c r="B435" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="C435" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="436" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A436" s="9">
+        <v>3503</v>
+      </c>
+      <c r="B436" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="C436" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="437" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A437" s="9">
+        <v>28573</v>
+      </c>
+      <c r="B437" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="C437" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="438" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A438" s="9">
+        <v>90885</v>
+      </c>
+      <c r="B438" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="C438" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="439" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A439" s="9">
+        <v>67263</v>
+      </c>
+      <c r="B439" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="C439" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="440" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A440" s="9">
+        <v>88303</v>
+      </c>
+      <c r="B440" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="C440" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="441" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A441" s="9">
+        <v>60969</v>
+      </c>
+      <c r="B441" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="C441" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="442" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A442" s="9">
+        <v>55889</v>
+      </c>
+      <c r="B442" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="C442" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="443" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A443" s="9">
+        <v>74716</v>
+      </c>
+      <c r="B443" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="C443" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="444" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A444" s="9">
+        <v>67227</v>
+      </c>
+      <c r="B444" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="C444" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="445" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A445" s="9">
+        <v>74080</v>
+      </c>
+      <c r="B445" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="C445" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="446" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A446" s="9">
+        <v>79107</v>
+      </c>
+      <c r="B446" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="C446" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="447" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A447" s="9">
+        <v>75050</v>
+      </c>
+      <c r="B447" s="9" t="s">
+        <v>425</v>
+      </c>
+      <c r="C447" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="448" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A448" s="9">
+        <v>82466</v>
+      </c>
+      <c r="B448" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="C448" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="449" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A449" s="9">
+        <v>745822</v>
+      </c>
+      <c r="B449" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="C449" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="450" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A450" s="9">
+        <v>84842</v>
+      </c>
+      <c r="B450" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="C450" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="451" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A451" s="9">
+        <v>81078</v>
+      </c>
+      <c r="B451" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="C451" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="452" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A452" s="9">
+        <v>82428</v>
+      </c>
+      <c r="B452" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="C452" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="453" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A453" s="9">
+        <v>81236</v>
+      </c>
+      <c r="B453" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="C453" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="454" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A454" s="9">
+        <v>59101</v>
+      </c>
+      <c r="B454" s="9" t="s">
+        <v>432</v>
+      </c>
+      <c r="C454" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="455" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A455" s="9">
+        <v>78677</v>
+      </c>
+      <c r="B455" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="C455" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="456" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A456" s="9">
+        <v>23302</v>
+      </c>
+      <c r="B456" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="C456" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="457" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A457" s="9">
+        <v>85884</v>
+      </c>
+      <c r="B457" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="C457" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="458" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A458" s="9">
+        <v>49579</v>
+      </c>
+      <c r="B458" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="C458" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="459" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A459" s="9">
+        <v>82381</v>
+      </c>
+      <c r="B459" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="C459" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="460" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A460" s="9">
+        <v>92725</v>
+      </c>
+      <c r="B460" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="C460" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="461" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A461" s="9">
+        <v>53470</v>
+      </c>
+      <c r="B461" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="C461" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="462" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A462" s="9">
+        <v>4522</v>
+      </c>
+      <c r="B462" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="C462" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="463" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A463" s="9">
+        <v>74023</v>
+      </c>
+      <c r="B463" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="C463" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="464" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A464" s="9">
+        <v>92743</v>
+      </c>
+      <c r="B464" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="C464" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="465" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A465" s="9">
+        <v>21483</v>
+      </c>
+      <c r="B465" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="C465" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="466" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A466" s="9">
+        <v>80802</v>
+      </c>
+      <c r="B466" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="C466" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="467" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A467" s="9">
+        <v>91036</v>
+      </c>
+      <c r="B467" s="9" t="s">
+        <v>406</v>
+      </c>
+      <c r="C467" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="468" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A468" s="9">
+        <v>1188</v>
+      </c>
+      <c r="B468" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="C468" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="469" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A469" s="9">
+        <v>84778</v>
+      </c>
+      <c r="B469" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="C469" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="470" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A470" s="9">
+        <v>18096</v>
+      </c>
+      <c r="B470" s="9" t="s">
+        <v>409</v>
+      </c>
+      <c r="C470" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="471" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A471" s="9">
+        <v>17699</v>
+      </c>
+      <c r="B471" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="C471" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="472" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A472" s="9">
+        <v>65983</v>
+      </c>
+      <c r="B472" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="C472" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="473" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A473" s="9">
+        <v>90949</v>
+      </c>
+      <c r="B473" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="C473" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="474" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A474" s="9">
+        <v>8784</v>
+      </c>
+      <c r="B474" s="9" t="s">
+        <v>413</v>
+      </c>
+      <c r="C474" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="475" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A475" s="9">
+        <v>3503</v>
+      </c>
+      <c r="B475" s="9" t="s">
+        <v>414</v>
+      </c>
+      <c r="C475" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="476" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A476" s="9">
+        <v>28573</v>
+      </c>
+      <c r="B476" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="C476" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="477" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A477" s="9">
+        <v>90885</v>
+      </c>
+      <c r="B477" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="C477" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="478" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A478" s="9">
+        <v>67263</v>
+      </c>
+      <c r="B478" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="C478" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="479" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A479" s="9">
+        <v>88303</v>
+      </c>
+      <c r="B479" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="C479" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="480" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A480" s="9">
+        <v>60969</v>
+      </c>
+      <c r="B480" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="C480" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="481" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A481" s="9">
+        <v>55889</v>
+      </c>
+      <c r="B481" s="9" t="s">
+        <v>420</v>
+      </c>
+      <c r="C481" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="482" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A482" s="9">
+        <v>74716</v>
+      </c>
+      <c r="B482" s="9" t="s">
+        <v>421</v>
+      </c>
+      <c r="C482" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="483" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A483" s="9">
+        <v>67227</v>
+      </c>
+      <c r="B483" s="9" t="s">
+        <v>422</v>
+      </c>
+      <c r="C483" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="484" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A484" s="9">
+        <v>74080</v>
+      </c>
+      <c r="B484" s="9" t="s">
+        <v>423</v>
+      </c>
+      <c r="C484" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="485" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A485" s="9">
+        <v>79107</v>
+      </c>
+      <c r="B485" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="C485" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="486" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A486" s="9">
+        <v>75050</v>
+      </c>
+      <c r="B486" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="C486" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="487" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A487" s="9">
+        <v>82466</v>
+      </c>
+      <c r="B487" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="C487" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="488" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A488" s="9">
+        <v>745822</v>
+      </c>
+      <c r="B488" s="9" t="s">
+        <v>427</v>
+      </c>
+      <c r="C488" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="489" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A489" s="9">
+        <v>84842</v>
+      </c>
+      <c r="B489" s="9" t="s">
+        <v>428</v>
+      </c>
+      <c r="C489" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="490" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A490" s="9">
+        <v>81078</v>
+      </c>
+      <c r="B490" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="C490" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="491" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A491" s="9">
+        <v>82428</v>
+      </c>
+      <c r="B491" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="C491" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="492" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A492" s="9">
+        <v>81236</v>
+      </c>
+      <c r="B492" s="9" t="s">
+        <v>431</v>
+      </c>
+      <c r="C492" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="493" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A493" s="9">
+        <v>81575</v>
+      </c>
+      <c r="B493" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="C493" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="494" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A494" s="9">
+        <v>89262</v>
+      </c>
+      <c r="B494" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="C494" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="495" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A495">
+        <v>80691</v>
+      </c>
+      <c r="B495" t="s">
+        <v>443</v>
+      </c>
+      <c r="C495" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="496" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A496">
+        <v>86544</v>
+      </c>
+      <c r="B496" t="s">
+        <v>445</v>
+      </c>
+      <c r="C496" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="497" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A497">
+        <v>79694</v>
+      </c>
+      <c r="B497" t="s">
+        <v>446</v>
+      </c>
+      <c r="C497" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="498" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A498" s="10">
+        <v>47262</v>
+      </c>
+      <c r="B498" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="C498" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="499" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A499" s="10">
+        <v>78258</v>
+      </c>
+      <c r="B499" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="C499" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="500" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A500">
+        <v>88581</v>
+      </c>
+      <c r="B500" t="s">
+        <v>452</v>
+      </c>
+      <c r="C500" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="501" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A501">
+        <v>26492</v>
+      </c>
+      <c r="B501" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="C501" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="502" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B502" s="11" t="s">
+        <v>455</v>
+      </c>
+      <c r="C502" t="s">
+        <v>456</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>